<commit_message>
data: sync 06.07 numbers into GR/EN workbooks (Ilioupoli project + 15 rows, 2 decimals)
</commit_message>
<xml_diff>
--- a/LA_Budgeting_EN.xlsx
+++ b/LA_Budgeting_EN.xlsx
@@ -540,14 +540,14 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1558,7 +1558,11 @@
         </is>
       </c>
       <c r="F5" s="40" t="n"/>
-      <c r="H5" s="43" t="n"/>
+      <c r="H5" s="33" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
       <c r="I5" s="34">
         <f>IF($H5="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H5,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1573,24 +1577,24 @@
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="43" t="inlineStr">
         <is>
           <t>📊  Grand Total Budget</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n"/>
-      <c r="C6" s="45" t="n"/>
+      <c r="B6" s="44" t="n"/>
+      <c r="C6" s="44" t="n"/>
       <c r="D6" s="15">
         <f>D4+D5</f>
         <v/>
       </c>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="45" t="inlineStr">
         <is>
           <t>All projects (paid + upcoming)</t>
         </is>
       </c>
-      <c r="F6" s="45" t="n"/>
-      <c r="H6" s="43" t="n"/>
+      <c r="F6" s="44" t="n"/>
+      <c r="H6" s="46" t="n"/>
       <c r="I6" s="34">
         <f>IF($H6="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H6,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1611,7 +1615,7 @@
       <c r="D7" s="21" t="n"/>
       <c r="E7" s="21" t="n"/>
       <c r="F7" s="21" t="n"/>
-      <c r="H7" s="43" t="n"/>
+      <c r="H7" s="46" t="n"/>
       <c r="I7" s="34">
         <f>IF($H7="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H7,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1632,7 +1636,7 @@
       <c r="D8" s="21" t="n"/>
       <c r="E8" s="21" t="n"/>
       <c r="F8" s="21" t="n"/>
-      <c r="H8" s="43" t="n"/>
+      <c r="H8" s="46" t="n"/>
       <c r="I8" s="34">
         <f>IF($H8="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H8,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1653,7 +1657,7 @@
       <c r="D9" s="21" t="n"/>
       <c r="E9" s="21" t="n"/>
       <c r="F9" s="21" t="n"/>
-      <c r="H9" s="43" t="n"/>
+      <c r="H9" s="46" t="n"/>
       <c r="I9" s="34">
         <f>IF($H9="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H9,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1674,7 +1678,7 @@
       <c r="D10" s="21" t="n"/>
       <c r="E10" s="21" t="n"/>
       <c r="F10" s="21" t="n"/>
-      <c r="H10" s="43" t="n"/>
+      <c r="H10" s="46" t="n"/>
       <c r="I10" s="34">
         <f>IF($H10="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H10,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1695,7 +1699,7 @@
       <c r="D11" s="21" t="n"/>
       <c r="E11" s="21" t="n"/>
       <c r="F11" s="21" t="n"/>
-      <c r="H11" s="43" t="n"/>
+      <c r="H11" s="46" t="n"/>
       <c r="I11" s="34">
         <f>IF($H11="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H11,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1740,7 +1744,7 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="H12" s="43" t="n"/>
+      <c r="H12" s="46" t="n"/>
       <c r="I12" s="34">
         <f>IF($H12="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H12,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1779,7 +1783,7 @@
         <v>5000</v>
       </c>
       <c r="F13" s="53" t="inlineStr"/>
-      <c r="H13" s="43" t="n"/>
+      <c r="H13" s="46" t="n"/>
       <c r="I13" s="34">
         <f>IF($H13="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H13,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -1818,7 +1822,7 @@
         <v>1000</v>
       </c>
       <c r="F14" s="53" t="inlineStr"/>
-      <c r="H14" s="43" t="n"/>
+      <c r="H14" s="46" t="n"/>
       <c r="I14" s="34">
         <f>IF($H14="","",SUMIFS(Table_Exp[Amount],Table_Exp[Project],$H14,Table_Exp[Status],"Paid"))</f>
         <v/>
@@ -2342,124 +2346,392 @@
       <c r="F32" s="53" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="58" t="n"/>
-      <c r="B33" s="59" t="n"/>
-      <c r="C33" s="58" t="n"/>
-      <c r="D33" s="58" t="n"/>
-      <c r="E33" s="60" t="n"/>
-      <c r="F33" s="59" t="n"/>
+      <c r="A33" s="48" t="inlineStr">
+        <is>
+          <t>Lazaraki 5</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Common Expenses</t>
+        </is>
+      </c>
+      <c r="C33" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D33" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E33" s="52" t="n">
+        <v>210.24</v>
+      </c>
+      <c r="F33" s="53" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="58" t="n"/>
-      <c r="B34" s="59" t="n"/>
-      <c r="C34" s="58" t="n"/>
-      <c r="D34" s="58" t="n"/>
-      <c r="E34" s="60" t="n"/>
-      <c r="F34" s="59" t="n"/>
+      <c r="A34" s="57" t="inlineStr">
+        <is>
+          <t>Agiou Konstantinou</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Nektaria Advance</t>
+        </is>
+      </c>
+      <c r="C34" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D34" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E34" s="52" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F34" s="53" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="58" t="n"/>
-      <c r="B35" s="59" t="n"/>
-      <c r="C35" s="58" t="n"/>
-      <c r="D35" s="58" t="n"/>
-      <c r="E35" s="60" t="n"/>
-      <c r="F35" s="59" t="n"/>
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>Agiou Konstantinou</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Tax settlement reinstatement</t>
+        </is>
+      </c>
+      <c r="C35" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D35" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E35" s="52" t="n">
+        <v>1428.56</v>
+      </c>
+      <c r="F35" s="53" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="58" t="n"/>
-      <c r="B36" s="59" t="n"/>
-      <c r="C36" s="58" t="n"/>
-      <c r="D36" s="58" t="n"/>
-      <c r="E36" s="60" t="n"/>
-      <c r="F36" s="59" t="n"/>
+      <c r="A36" s="48" t="inlineStr">
+        <is>
+          <t>Lazaraki 5</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>Elevator common expenses</t>
+        </is>
+      </c>
+      <c r="C36" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D36" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E36" s="52" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="F36" s="53" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="58" t="n"/>
-      <c r="B37" s="59" t="n"/>
-      <c r="C37" s="58" t="n"/>
-      <c r="D37" s="58" t="n"/>
-      <c r="E37" s="60" t="n"/>
-      <c r="F37" s="59" t="n"/>
+      <c r="A37" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Architectural TAF</t>
+        </is>
+      </c>
+      <c r="C37" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D37" s="51" t="inlineStr">
+        <is>
+          <t>Optima Bank</t>
+        </is>
+      </c>
+      <c r="E37" s="52" t="n"/>
+      <c r="F37" s="53" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="58" t="n"/>
-      <c r="B38" s="59" t="n"/>
-      <c r="C38" s="58" t="n"/>
-      <c r="D38" s="58" t="n"/>
-      <c r="E38" s="60" t="n"/>
-      <c r="F38" s="59" t="n"/>
+      <c r="A38" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>Rteco structural &amp; mechanical permit</t>
+        </is>
+      </c>
+      <c r="C38" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D38" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E38" s="52" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F38" s="53" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="58" t="n"/>
-      <c r="B39" s="59" t="n"/>
-      <c r="C39" s="58" t="n"/>
-      <c r="D39" s="58" t="n"/>
-      <c r="E39" s="60" t="n"/>
-      <c r="F39" s="59" t="n"/>
+      <c r="A39" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>Vaso purchase advance</t>
+        </is>
+      </c>
+      <c r="C39" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D39" s="51" t="inlineStr">
+        <is>
+          <t>Optima Bank</t>
+        </is>
+      </c>
+      <c r="E39" s="52" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F39" s="53" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="58" t="n"/>
-      <c r="B40" s="59" t="n"/>
-      <c r="C40" s="58" t="n"/>
-      <c r="D40" s="58" t="n"/>
-      <c r="E40" s="60" t="n"/>
-      <c r="F40" s="59" t="n"/>
+      <c r="A40" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>Notary purchase contract</t>
+        </is>
+      </c>
+      <c r="C40" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D40" s="51" t="inlineStr">
+        <is>
+          <t>Optima Bank</t>
+        </is>
+      </c>
+      <c r="E40" s="52" t="n">
+        <v>1253.16</v>
+      </c>
+      <c r="F40" s="53" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="58" t="n"/>
-      <c r="B41" s="59" t="n"/>
-      <c r="C41" s="58" t="n"/>
-      <c r="D41" s="58" t="n"/>
-      <c r="E41" s="60" t="n"/>
-      <c r="F41" s="59" t="n"/>
+      <c r="A41" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Lawyer</t>
+        </is>
+      </c>
+      <c r="C41" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D41" s="51" t="inlineStr">
+        <is>
+          <t>Optima Bank</t>
+        </is>
+      </c>
+      <c r="E41" s="52" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F41" s="53" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="58" t="n"/>
-      <c r="B42" s="59" t="n"/>
-      <c r="C42" s="58" t="n"/>
-      <c r="D42" s="58" t="n"/>
-      <c r="E42" s="60" t="n"/>
-      <c r="F42" s="59" t="n"/>
+      <c r="A42" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>Land Registry</t>
+        </is>
+      </c>
+      <c r="C42" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D42" s="51" t="inlineStr">
+        <is>
+          <t>Optima Bank</t>
+        </is>
+      </c>
+      <c r="E42" s="52" t="n">
+        <v>749.5</v>
+      </c>
+      <c r="F42" s="53" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="58" t="n"/>
-      <c r="B43" s="59" t="n"/>
-      <c r="C43" s="58" t="n"/>
-      <c r="D43" s="58" t="n"/>
-      <c r="E43" s="60" t="n"/>
-      <c r="F43" s="59" t="n"/>
+      <c r="A43" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Purchase Transfer Tax (FMA)</t>
+        </is>
+      </c>
+      <c r="C43" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D43" s="51" t="inlineStr">
+        <is>
+          <t>Optima Bank</t>
+        </is>
+      </c>
+      <c r="E43" s="52" t="n">
+        <v>3708</v>
+      </c>
+      <c r="F43" s="53" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="58" t="n"/>
-      <c r="B44" s="59" t="n"/>
-      <c r="C44" s="58" t="n"/>
-      <c r="D44" s="58" t="n"/>
-      <c r="E44" s="60" t="n"/>
-      <c r="F44" s="59" t="n"/>
+      <c r="A44" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>Legalizations</t>
+        </is>
+      </c>
+      <c r="C44" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D44" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E44" s="52" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F44" s="53" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="58" t="n"/>
-      <c r="B45" s="59" t="n"/>
-      <c r="C45" s="58" t="n"/>
-      <c r="D45" s="58" t="n"/>
-      <c r="E45" s="60" t="n"/>
-      <c r="F45" s="59" t="n"/>
+      <c r="A45" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B45" s="49" t="inlineStr">
+        <is>
+          <t>Height acceptance notary</t>
+        </is>
+      </c>
+      <c r="C45" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D45" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E45" s="52" t="n">
+        <v>450</v>
+      </c>
+      <c r="F45" s="53" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="58" t="n"/>
-      <c r="B46" s="59" t="n"/>
-      <c r="C46" s="58" t="n"/>
-      <c r="D46" s="58" t="n"/>
-      <c r="E46" s="60" t="n"/>
-      <c r="F46" s="59" t="n"/>
+      <c r="A46" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>Topographic survey</t>
+        </is>
+      </c>
+      <c r="C46" s="50" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D46" s="51" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E46" s="52" t="n">
+        <v>300</v>
+      </c>
+      <c r="F46" s="53" t="inlineStr"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="58" t="n"/>
-      <c r="B47" s="59" t="n"/>
-      <c r="C47" s="58" t="n"/>
-      <c r="D47" s="58" t="n"/>
-      <c r="E47" s="60" t="n"/>
-      <c r="F47" s="59" t="n"/>
+      <c r="A47" s="57" t="inlineStr">
+        <is>
+          <t>Ilioupoli</t>
+        </is>
+      </c>
+      <c r="B47" s="49" t="inlineStr">
+        <is>
+          <t>Vaso purchase completion</t>
+        </is>
+      </c>
+      <c r="C47" s="56" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="D47" s="51" t="inlineStr">
+        <is>
+          <t>Optima Bank</t>
+        </is>
+      </c>
+      <c r="E47" s="52" t="n">
+        <v>70000</v>
+      </c>
+      <c r="F47" s="53" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="58" t="n"/>
@@ -2742,8 +3014,8 @@
         <f>SUM(B5:B8)+SUM(B23:B32)</f>
         <v/>
       </c>
-      <c r="C10" s="45" t="n"/>
-      <c r="D10" s="45" t="n"/>
+      <c r="C10" s="44" t="n"/>
+      <c r="D10" s="44" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="21" t="n"/>
@@ -2816,8 +3088,8 @@
         <f>SUM(B14:B15)+SUM(B36:B40)</f>
         <v/>
       </c>
-      <c r="C17" s="45" t="n"/>
-      <c r="D17" s="45" t="n"/>
+      <c r="C17" s="44" t="n"/>
+      <c r="D17" s="44" t="n"/>
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="A18" s="21" t="n"/>
@@ -3053,7 +3325,7 @@
           <t>What each tab does:</t>
         </is>
       </c>
-      <c r="D4" s="45" t="n"/>
+      <c r="D4" s="44" t="n"/>
     </row>
     <row r="5" ht="37" customHeight="1">
       <c r="A5" s="74" t="n"/>
@@ -3400,7 +3672,7 @@
       <c r="D42" s="86" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="45" t="n"/>
+      <c r="A43" s="44" t="n"/>
       <c r="B43" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  Blue background = calculated formula — do not edit</t>

</xml_diff>